<commit_message>
Remove unnecessary excel page
</commit_message>
<xml_diff>
--- a/3-Workflow-Analysis/Workflow_Analysis.xlsx
+++ b/3-Workflow-Analysis/Workflow_Analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marci/Desktop/Creative-Visual-Design-Accessibility-Tools/Research/Workflow Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marci/Documents/GitHub/design-accessibility-tools/3-Workflow-Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C47B360-5EA1-6C4A-95C6-38F451755C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230123F9-E042-5C48-858C-84ACCB54D0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" firstSheet="2" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,8 +24,7 @@
     <sheet name="Video-8-Sample-1" sheetId="9" r:id="rId9"/>
     <sheet name="Video-9-Sample-1" sheetId="10" r:id="rId10"/>
     <sheet name="Video-10-Sample-1" sheetId="11" r:id="rId11"/>
-    <sheet name="total_data" sheetId="12" r:id="rId12"/>
-    <sheet name="_lists" sheetId="13" r:id="rId13"/>
+    <sheet name="_lists" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1589,6 +1588,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6649D996-6833-C548-BBDE-C83189B87AE7}">
+  <we:reference id="93533c7f-4dc5-468f-aba4-1c008e1a7ac8" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200003101" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U200"/>
@@ -9701,76 +9720,6 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="B2:F22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B2">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B3">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B4">
-        <v>67</v>
-      </c>
-      <c r="E4">
-        <f>SUM(B2:B4)</f>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B5">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B6">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B7">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B12">
-        <f>SUM(B2:B7)</f>
-        <v>242</v>
-      </c>
-    </row>
-    <row r="21" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D21">
-        <f>36 + 17.5 + 44.75 + 92 + 60 + 55.5 + 120 + 58 + 25.25 + 60 + 41 + 60 + 18 + 60 + 19.75</f>
-        <v>767.75</v>
-      </c>
-      <c r="F21">
-        <f>D21-D22</f>
-        <v>690.97500000000002</v>
-      </c>
-    </row>
-    <row r="22" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D22">
-        <f>D21*0.1</f>
-        <v>76.775000000000006</v>
-      </c>
-      <c r="F22">
-        <f>F21/60</f>
-        <v>11.516250000000001</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>